<commit_message>
Add review for 127156021_ASHLEY (Q23)
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results.xlsx
+++ b/G2_Coding_Challenge_Review_Results.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2032,6 +2032,60 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>127156021_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Q23</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Correct O(n) set-based sequence-start detection matching AI focus guidance; Both provided examples pass (length 4, length 5) plus an additional manual test with duplicates</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>No negative-number test recorded despite being a stated edge case; No comments or error handling; File is misleadingly named 'Longest_common_subsequence.py' though it correctly solves Longest Consecutive Sequence</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2064,7 +2118,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -2074,7 +2128,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74.38</v>
+        <v>74.95999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -2111,7 +2165,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Mark AI Used as Yes for folders containing a README.md
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results.xlsx
+++ b/G2_Coding_Challenge_Review_Results.xlsx
@@ -851,7 +851,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Correct AI Used rule: exclude README.md, factor in other markdown files
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results.xlsx
+++ b/G2_Coding_Challenge_Review_Results.xlsx
@@ -851,7 +851,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>No negative-number test recorded despite being a stated edge case; No comments or error handling; File is misleadingly named 'Longest_common_subsequence.py' though it correctly solves Longest Consecutive Sequence</t>
+          <t>No negative-number test recorded despite being a stated edge case; No comments or error handling; File is misleadingly named 'Longest_common_subsequence.py' though it correctly solves Longest Consecutive Sequence; Contains an extra OUTPUT.md file documenting manual test runs, alongside the problem-statement markdown</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Add review for 127179060_ASHLEY (Q09) - non-runnable due to invalid comment syntax
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results.xlsx
+++ b/G2_Coding_Challenge_Review_Results.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2086,6 +2086,64 @@
       </c>
       <c r="N28" s="3" t="inlineStr"/>
     </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>127179060_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Q09</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Correct hashmap-based first-seen-index design with early exit on second occurrence, matching the expected algorithm</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: code uses '//' (C/Java-style) instead of '#' for comments on lines 1 and 3, causing a Python SyntaxError - the submitted file does not run as-is; results.txt transcript shows input prompts ('enter no of elements') that do not exist anywhere in the submitted code, indicating the recorded test evidence does not correspond to the actual submitted file; No error handling or input validation</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: Non-runnable submission (SyntaxError from // comments); Test evidence mismatch with submitted code</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2118,7 +2176,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -2128,7 +2186,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74.95999999999999</v>
+        <v>73.56999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -2205,7 +2263,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deep-dive review: correct 127156039_ASHLEY score for non-runnable IndentationError bug
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results.xlsx
+++ b/G2_Coding_Challenge_Review_Results.xlsx
@@ -60,12 +60,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
@@ -74,6 +68,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFD966"/>
         <bgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -620,13 +620,13 @@
         <v>15</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>15</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
@@ -640,10 +640,14 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Correct on example and all edge cases (1x1, single row, single column); Elegant border-sum condition avoids double counting corners; Comprehensive test output shown</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr"/>
+          <t>Matches Example 1 (3x4-&gt;65) and correctly handles the 1x1 mandatory edge case (42-&gt;42); Elegant single border-sum condition (i==0 or i==r-1 or j==0 or j==c-1) avoids double counting corners; Code-inspection confirms the condition also correctly handles single-row/single-column matrices even though untested</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Mandatory edge case 'single row or single column' was never exercised in the submitted test evidence (Output.png) - the third run (3x5) is just another normal-size matrix, not an edge case; No automated/assert-based tests, only manual terminal runs; No input validation or comments</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -827,26 +831,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>9</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -856,17 +860,17 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Correct email validation and metrics math; Matches example output exactly</t>
+          <t>Correct email validation logic (id required, exactly one '@', non-empty local/domain parts) and correct duplicate-tracking design using dict keyed by id; Design intent is correct: last-write-wins per id, matching the expected 'valid/rejected/duplicates_removed' metrics</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Indentation formatting oddity in notebook JSON; No additional edge-case tests beyond one example; Missing comments</t>
+          <t>CRITICAL: extracted source is non-runnable as submitted - confirmed via execution, raises 'IndentationError: unexpected indent' on the 'record=records[id]' line because it sits outside the for-loop (the preceding 'duplicates_removed=...' line is unindented, closing the loop early) while the print statements below it are still indented as if inside the loop; The single stdin/stdout transcript captured in the notebook could not have been produced by this exact code given the IndentationError, indicating the recorded output does not match the submitted source; No automated tests, only one manual run</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Limited test coverage</t>
+          <t>CRITICAL: Non-runnable submission (IndentationError); Test evidence mismatch with submitted code</t>
         </is>
       </c>
     </row>
@@ -1003,10 +1007,10 @@
       <c r="H9" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1061,10 +1065,10 @@
       <c r="H10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="I10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1119,10 +1123,10 @@
       <c r="H11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I11" s="7" t="n">
+      <c r="I11" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -1227,10 +1231,10 @@
       <c r="H13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1447,10 +1451,10 @@
       <c r="H17" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I17" s="7" t="n">
+      <c r="I17" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -1505,10 +1509,10 @@
       <c r="H18" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="7" t="n">
         <v>75</v>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1721,10 +1725,10 @@
       <c r="H22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="I22" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -1891,10 +1895,10 @@
       <c r="H25" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I25" s="6" t="n">
+      <c r="I25" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -2003,10 +2007,10 @@
       <c r="H27" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="I27" s="6" t="n">
+      <c r="I27" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -2115,10 +2119,10 @@
       <c r="H29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I29" s="6" t="n">
+      <c r="I29" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
@@ -2186,7 +2190,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>73.56999999999999</v>
+        <v>71.75</v>
       </c>
     </row>
     <row r="5">
@@ -2233,7 +2237,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2263,7 +2267,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine 127156063_ASHLEY Q09 review wording after re-validation
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results.xlsx
+++ b/G2_Coding_Challenge_Review_Results.xlsx
@@ -1080,17 +1080,17 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Code is syntactically clean</t>
+          <t>Coding Challenge 9.md (earliest second-occurrence distance) problem statement is present in the folder</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>CRITICAL: Wrong problem solved (Q10 code submitted instead of Q09); No earliest-second-occurrence logic present</t>
+          <t>CRITICAL: No code addressing Q09 was submitted - the folder's only notebook (Coding_answer.ipynb) contains a single code cell, and that cell fully implements the unrelated Q10 event-counting-by-date problem instead; No first-seen-index tracking, no distance calculation, no 'NONE' handling, no test evidence for Q09 exists anywhere</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>CRITICAL: Wrong problem solved</t>
+          <t>CRITICAL: No submission for this question (Q10 code present instead)</t>
         </is>
       </c>
     </row>

</xml_diff>